<commit_message>
style(kit-datos): aplicar estilo visual corporativo profesional al archivo Excel RAT
</commit_message>
<xml_diff>
--- a/api/assets/kit_datos_files/4_Registro_Actividades_Tratamiento_RAT_Ley_21719.xlsx
+++ b/api/assets/kit_datos_files/4_Registro_Actividades_Tratamiento_RAT_Ley_21719.xlsx
@@ -12,7 +12,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -20,16 +20,124 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00E2E8F0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000F172A"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="000284C7"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00059669"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00BE123C"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000369A1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00334155"/>
+      <sz val="9.5"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F172A"/>
+        <bgColor rgb="000F172A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E293B"/>
+        <bgColor rgb="001E293B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F9FF"/>
+        <bgColor rgb="00F0F9FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000284C7"/>
+        <bgColor rgb="000284C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -37,12 +145,75 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -460,472 +631,513 @@
     <col width="50.83203125" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>REGISTRO DE ACTIVIDADES DE TRATAMIENTO DE DATOS PERSONALES (RAT)</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Conforme al Artículo 14 ter de la Ley N° 21.719 - Agencia de Protección de Datos Personales (APDP) Chile</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Inventario Oficial Obligatorio conforme al Artículo 14 ter de la Ley N° 21.719 - Agencia de Protección de Datos Personales (APDP) Chile</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Empresa Responsable:</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>[NOMBRE DE TU EMPRESA]</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>RUT:</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>[RUT EMPRESA]</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Fecha de Emisión / Actualización:</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Septiembre de 2026</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
+      <c r="J3" s="4" t="n"/>
+    </row>
+    <row r="4" ht="10" customHeight="1"/>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Código RAT</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Área / Proceso</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Categoría de Datos Personales</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Titulares Afectados</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Finalidad del Tratamiento</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Base Legal de Licitud (Art. 13)</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>¿Datos Sensibles? (Art. 12)</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Destinatarios / Encargados Externos</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Plazo de Conservación</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Medidas de Seguridad Aplicadas (Art. 14 bis)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="55" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>RAT-01</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Recursos Humanos</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Nombre, RUT, sueldos, cuentas bancarias, domicilio, cotizaciones</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>Trabajadores activos y extrabajadores</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Liquidaciones de sueldo, transferencias bancarias, retención judicial pensión alimentos y pago en Previred</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Cumplimiento contractual y mandato legal Código del Trabajo (Arts. 154 bis y ter)</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>Banco pagador, Software de Nómina, Previred, Dirección del Trabajo (portal Mi DT)</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Hasta 5 años tras término relación laboral (Arts. 480 y 510 CT) y 6 años respaldo tributario/previsional (Art. 200 CTrib)</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="8" t="inlineStr">
         <is>
           <t>Servidor cifrado, control de accesos con doble factor (2FA) y claves individuales</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="55" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>RAT-02</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Recursos Humanos</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Licencias médicas, diagnósticos de salud, exámenes ocupacionales</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Trabajadores dependientes</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Tramitación legal de subsidios por incapacidad ante COMPIN/Isapre y prevención de riesgos (Ley 16.744)</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="12" t="inlineStr">
         <is>
           <t>Obligación legal previsional y de salud pública (DFL 1, Min. Salud)</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="13" t="inlineStr">
         <is>
           <t>SÍ (Salud)</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="12" t="inlineStr">
         <is>
           <t>COMPIN, Isapres, Mutualidades de Seguridad. Prohibido acceso a jefaturas directas</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="12" t="inlineStr">
         <is>
           <t>5 años desde su tramitación legal</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" s="12" t="inlineStr">
         <is>
           <t>Carpeta digital confidencial con acceso restringido exclusivo a Encargado RRHH</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="8" ht="55" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>RAT-03</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Operaciones &amp; RRHH</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Patrones biométricos encriptados (algoritmo huella digital o rostro)</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Personal afecto a control de asistencia</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Registro y control de jornada ordinaria y extraordinaria de trabajo</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Cumplimiento legal Art. 33 Código del Trabajo y Res. Exenta N° 38/2024 de la Dirección del Trabajo</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="14" t="inlineStr">
         <is>
           <t>SÍ (Biométrico)</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>Proveedor del reloj control de asistencia homologado y certificado ante la DT</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>Durante la vigencia del contrato de trabajo</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>Plantillas algorítmicas encriptadas sin fotos reales. Alternativa no biométrica obligatoria garantizada</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="9" ht="55" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>RAT-04</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Ventas &amp; Facturación</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Nombre completo, RUT, dirección de entrega, correo, teléfono</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Clientes compradores</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Emisión de boletas y facturas electrónicas, cobranza y despacho logístico de productos</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>Ejecución contractual de compraventa y obligación tributaria ante el SII (Código Tributario)</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" s="12" t="inlineStr">
         <is>
           <t>Servicio de Impuestos Internos (SII), Pasarela de Pago, Couriers logísticos de despacho</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" s="12" t="inlineStr">
         <is>
           <t>6 años (Plazo de prescripción tributaria según normas del SII)</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J9" s="12" t="inlineStr">
         <is>
           <t>Cifrado TLS/SSL en web, pasarela de pago certificada PCI-DSS compliance</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="10" ht="55" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>RAT-05</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Marketing &amp; Comercial</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Nombre, correo electrónico, teléfono celular</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Prospectos comerciales y clientes registrados</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Envío de promociones comerciales, novedades del servicio y cotizaciones solicitadas</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>Consentimiento previo, expreso e informado del titular (Art. 13 letra c)</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>Plataforma de Email Marketing / CRM en la nube con contrato DPA firmado</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I10" s="8" t="inlineStr">
         <is>
           <t>Hasta que el titular revoque su consentimiento (Derecho de Oposición ARCOP)</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J10" s="8" t="inlineStr">
         <is>
           <t>Enlace directo y gratuito de desuscripción automática (opt-out) en cada comunicación</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="11" ht="55" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>RAT-06</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Seguridad de Instalaciones</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>Imágenes y grabaciones de video en circuito cerrado (CCTV)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Colaboradores, clientes, proveedores y visitantes</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Seguridad física de las instalaciones, control de accesos y prevención de delitos</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>Interés legítimo del responsable en la seguridad patrimonial y física (Art. 13 letra e)</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="15" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>Tribunales de Justicia o Ministerio Público (exclusivamente ante orden judicial formal)</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I11" s="12" t="inlineStr">
         <is>
           <t>30 días continuos (salvo investigación judicial o policial en curso)</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J11" s="12" t="inlineStr">
         <is>
           <t>Sobreescritura cíclica automática cada 30 días, servidor de video DVR bajo llave física</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>INSTRUCCIONES OFICIALES DE CUMPLIMIENTO (LEY N° 21.719):</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>1. Obligatoriedad Legal:</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>Conforme al Artículo 14 ter de la Ley 21.719, toda empresa que trate datos personales debe mantener este inventario actualizado.</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+      <c r="E14" s="19" t="n"/>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="19" t="n"/>
+      <c r="H14" s="19" t="n"/>
+      <c r="I14" s="19" t="n"/>
+      <c r="J14" s="19" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>2. Exhibición Fiscalizadora:</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>Este documento es lo primero que exige la Agencia de Protección de Datos Personales (APDP) ante una auditoría.</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="19" t="n"/>
+      <c r="E15" s="19" t="n"/>
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="19" t="n"/>
+      <c r="H15" s="19" t="n"/>
+      <c r="I15" s="19" t="n"/>
+      <c r="J15" s="19" t="n"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>3. Sanción por Omisión:</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>No contar con el Registro RAT constituye Infracción Grave (Art. 35 N° 2) sancionable con multa de hasta 10.000 UTM (~ millones de pesos).</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="19" t="n"/>
+      <c r="E16" s="19" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="19" t="n"/>
+      <c r="H16" s="19" t="n"/>
+      <c r="I16" s="19" t="n"/>
+      <c r="J16" s="19" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>4. Personalización:</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>Puedes agregar nuevas filas si tu empresa realiza otras actividades de tratamiento (por ejemplo, encuestas o geolocalización GPS).</t>
         </is>
       </c>
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="19" t="n"/>
+      <c r="E17" s="19" t="n"/>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="19" t="n"/>
+      <c r="H17" s="19" t="n"/>
+      <c r="I17" s="19" t="n"/>
+      <c r="J17" s="19" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(excel): agregar pestana 1 de Guia Rapida Leeme Primero y limpiar metadata de fila 3
</commit_message>
<xml_diff>
--- a/api/assets/kit_datos_files/4_Registro_Actividades_Tratamiento_RAT_Ley_21719.xlsx
+++ b/api/assets/kit_datos_files/4_Registro_Actividades_Tratamiento_RAT_Ley_21719.xlsx
@@ -1,90 +1,104 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registro RAT Ley 21719" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📌 Guía Rápida" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📋 Registro RAT Oficial" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
-      <sz val="12"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00E2E8F0"/>
+      <color rgb="0094A3B8"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000284C7"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00334155"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00CBD5E1"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="10"/>
+      <color rgb="000284C7"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000F172A"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Calibri"/>
       <color rgb="000F172A"/>
-      <sz val="9.5"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Consolas"/>
       <b val="1"/>
       <color rgb="000284C7"/>
-      <sz val="10"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Calibri"/>
       <color rgb="00059669"/>
-      <sz val="9.5"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00BE123C"/>
-      <sz val="9.5"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="000F172A"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="000369A1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00334155"/>
-      <sz val="9.5"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="9">
@@ -97,43 +111,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000F172A"/>
-        <bgColor rgb="000F172A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001E293B"/>
-        <bgColor rgb="001E293B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F0F9FF"/>
-        <bgColor rgb="00F0F9FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000284C7"/>
-        <bgColor rgb="000284C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
-        <bgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
-        <bgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
   </fills>
@@ -163,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -171,54 +178,63 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -365,7 +381,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -400,7 +415,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -435,16 +449,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -566,46 +584,7 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -616,19 +595,134 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14.83203125" customWidth="1" min="1" max="1"/>
-    <col width="24.83203125" customWidth="1" min="2" max="2"/>
-    <col width="40.83203125" customWidth="1" min="3" max="3"/>
-    <col width="32.83203125" customWidth="1" min="4" max="4"/>
-    <col width="48.83203125" customWidth="1" min="5" max="5"/>
-    <col width="44.83203125" customWidth="1" min="6" max="6"/>
-    <col width="22.83203125" customWidth="1" min="7" max="7"/>
-    <col width="42.83203125" customWidth="1" min="8" max="8"/>
-    <col width="32.83203125" customWidth="1" min="9" max="9"/>
-    <col width="50.83203125" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>GUÍA RÁPIDA: ¿QUÉ ES EL REGISTRO RAT Y CÓMO USARLO EN TU EMPRESA?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Inventario Legal Obligatorio exigido por el Artículo 14 ter de la Ley N° 21.719 de Protección de Datos Personales en Chile</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>1. ¿QUÉ ES ESTE DOCUMENTO EN PALABRAS SIMPLES?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="126" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Así como el SII le exige a tu empresa llevar un 'Libro de Compras y Ventas' para fiscalizar el dinero, la nueva Ley N° 21.719 exige llevar un 'Libro de Datos Personales' (el RAT).
+Es simplemente un inventario oficial donde dejas por escrito qué información de personas manejas (empleados, clientes, proveedores), con quién la compartes (contador, bancos, Previred) y cuántos años la guardas antes de borrarla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2. ¿POR QUÉ LA AUTORIDAD (O UN ABOGADO) TE LO VA A PEDIR?</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="126" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Ante cualquier denuncia, inspección de la Dirección del Trabajo (DT) o auditoría de la nueva Agencia de Protección de Datos Personales (APDP), este Excel es el primer documento que te pedirán para comprobar si tu empresa cumple la ley.
+No tener el RAT constituye una 'Infracción Grave' que arriesga multas de hasta 10.000 UTM. Tenerlo al día demuestra diligencia y buena fe de la empresa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>3. ¿CÓMO SE USA ESTA PLANTILLA? (SOLO 3 PASOS):</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="144" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Paso 1: Ve a la siguiente pestaña: '📋 Registro RAT Oficial'.
+Paso 2: En la Fila 3, cambia [NOMBRE DE TU EMPRESA] por tu razón social y [RUT EMPRESA] por el RUT de tu negocio.
+Paso 3: ¡Listo! Las 6 filas ya vienen completamente rellenadas con los procesos habituales de una pyme chilena. No necesitas inventar nada. Guárdalo en tu computador o imprímelo para tu carpeta legal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>4. RESUMEN DE LAS 6 FILAS PRE-LLENADAS EN LA SIGUIENTE PESTAÑA:</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="234" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>• RAT-01 (Sueldos y RRHH): Nombres, RUTs y cuentas bancarias de trabajadores para pagar sueldos y cotizaciones en Previred.
+• RAT-02 (Licencias Médicas): Gestión confidencial de salud ante COMPIN/Isapre (prohibido compartir con jefaturas directas).
+• RAT-03 (Reloj Control con Huella): Control de asistencia biométrico con alternativa no biométrica obligatoria (Res. Exenta 38 DT).
+• RAT-04 (Ventas y Boletas): Datos de clientes para emitir facturas/boletas al SII y coordinar envíos por courier.
+• RAT-05 (Marketing y WhatsApp): Datos comerciales con opción obligatoria de desuscripción voluntaria (opt-out).
+• RAT-06 (Cámaras de Seguridad CCTV): Grabaciones en video de vigilancia que se sobreescriben automáticamente cada 30 días.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A8:H8"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -638,505 +732,422 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Inventario Oficial Obligatorio conforme al Artículo 14 ter de la Ley N° 21.719 - Agencia de Protección de Datos Personales (APDP) Chile</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Conforme al Artículo 14 ter de la Ley N° 21.719 - Agencia de Protección de Datos Personales (APDP) Chile</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Empresa Responsable:</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>[NOMBRE DE TU EMPRESA]</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>[NOMBRE DE TU EMPRESA / RAZÓN SOCIAL]</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>RUT:</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>[RUT EMPRESA]</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Fecha de Emisión / Actualización:</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="H3" s="7" t="n"/>
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>Septiembre de 2026</t>
         </is>
       </c>
-      <c r="G3" s="4" t="n"/>
-      <c r="H3" s="4" t="n"/>
-      <c r="I3" s="4" t="n"/>
-      <c r="J3" s="4" t="n"/>
-    </row>
-    <row r="4" ht="10" customHeight="1"/>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="J3" s="7" t="n"/>
+    </row>
+    <row r="4" ht="8" customHeight="1"/>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Código RAT</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Área / Proceso</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Categoría de Datos Personales</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>Titulares Afectados</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>Finalidad del Tratamiento</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="10" t="inlineStr">
         <is>
           <t>Base Legal de Licitud (Art. 13)</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="10" t="inlineStr">
         <is>
           <t>¿Datos Sensibles? (Art. 12)</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="10" t="inlineStr">
         <is>
           <t>Destinatarios / Encargados Externos</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" s="10" t="inlineStr">
         <is>
           <t>Plazo de Conservación</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J5" s="10" t="inlineStr">
         <is>
           <t>Medidas de Seguridad Aplicadas (Art. 14 bis)</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="55" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+    <row r="6" ht="54" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>RAT-01</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Recursos Humanos</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Nombre, RUT, sueldos, cuentas bancarias, domicilio, cotizaciones</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Nombre, RUT, sueldos, cuentas bancarias, cotizaciones, domicilio</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Trabajadores activos y extrabajadores</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Liquidaciones de sueldo, transferencias bancarias, retención judicial pensión alimentos y pago en Previred</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>Liquidaciones de sueldo, transferencias bancarias, retención judicial de pensión de alimentos y pago en Previred</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Cumplimiento contractual y mandato legal Código del Trabajo (Arts. 154 bis y ter)</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="H6" s="13" t="inlineStr">
         <is>
           <t>Banco pagador, Software de Nómina, Previred, Dirección del Trabajo (portal Mi DT)</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="I6" s="13" t="inlineStr">
         <is>
           <t>Hasta 5 años tras término relación laboral (Arts. 480 y 510 CT) y 6 años respaldo tributario/previsional (Art. 200 CTrib)</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr">
-        <is>
-          <t>Servidor cifrado, control de accesos con doble factor (2FA) y claves individuales</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="55" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>Servidor cifrado, control de accesos con doble factor (2FA) y claves individuales de usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="54" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>RAT-02</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>Recursos Humanos</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>Licencias médicas, diagnósticos de salud, exámenes ocupacionales</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>Trabajadores dependientes</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>Tramitación legal de subsidios por incapacidad ante COMPIN/Isapre y prevención de riesgos (Ley 16.744)</t>
         </is>
       </c>
-      <c r="F7" s="12" t="inlineStr">
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>Obligación legal previsional y de salud pública (DFL 1, Min. Salud)</t>
         </is>
       </c>
-      <c r="G7" s="13" t="inlineStr">
+      <c r="G7" s="18" t="inlineStr">
         <is>
           <t>SÍ (Salud)</t>
         </is>
       </c>
-      <c r="H7" s="12" t="inlineStr">
+      <c r="H7" s="17" t="inlineStr">
         <is>
           <t>COMPIN, Isapres, Mutualidades de Seguridad. Prohibido acceso a jefaturas directas</t>
         </is>
       </c>
-      <c r="I7" s="12" t="inlineStr">
+      <c r="I7" s="17" t="inlineStr">
         <is>
           <t>5 años desde su tramitación legal</t>
         </is>
       </c>
-      <c r="J7" s="12" t="inlineStr">
-        <is>
-          <t>Carpeta digital confidencial con acceso restringido exclusivo a Encargado RRHH</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="55" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="J7" s="17" t="inlineStr">
+        <is>
+          <t>Carpeta digital confidencial con acceso restringido exclusivo al Encargado de RRHH</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="54" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>RAT-03</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Operaciones &amp; RRHH</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Patrones biométricos encriptados (algoritmo huella digital o rostro)</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>Patrones biométricos encriptados (algoritmo matemático huella o rostro)</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>Personal afecto a control de asistencia</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>Registro y control de jornada ordinaria y extraordinaria de trabajo</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>Cumplimiento legal Art. 33 Código del Trabajo y Res. Exenta N° 38/2024 de la Dirección del Trabajo</t>
         </is>
       </c>
-      <c r="G8" s="14" t="inlineStr">
+      <c r="G8" s="19" t="inlineStr">
         <is>
           <t>SÍ (Biométrico)</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="H8" s="13" t="inlineStr">
         <is>
           <t>Proveedor del reloj control de asistencia homologado y certificado ante la DT</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr">
+      <c r="I8" s="13" t="inlineStr">
         <is>
           <t>Durante la vigencia del contrato de trabajo</t>
         </is>
       </c>
-      <c r="J8" s="8" t="inlineStr">
+      <c r="J8" s="13" t="inlineStr">
         <is>
           <t>Plantillas algorítmicas encriptadas sin fotos reales. Alternativa no biométrica obligatoria garantizada</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="55" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+    <row r="9" ht="54" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>RAT-04</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Ventas &amp; Facturación</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>Nombre completo, RUT, dirección de entrega, correo, teléfono</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>Clientes compradores</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>Emisión de boletas y facturas electrónicas, cobranza y despacho logístico de productos</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>Emisión de boletas y facturas electrónicas, cobranza y despacho logístico de pedidos</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>Ejecución contractual de compraventa y obligación tributaria ante el SII (Código Tributario)</t>
         </is>
       </c>
-      <c r="G9" s="15" t="inlineStr">
+      <c r="G9" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H9" s="12" t="inlineStr">
+      <c r="H9" s="17" t="inlineStr">
         <is>
           <t>Servicio de Impuestos Internos (SII), Pasarela de Pago, Couriers logísticos de despacho</t>
         </is>
       </c>
-      <c r="I9" s="12" t="inlineStr">
+      <c r="I9" s="17" t="inlineStr">
         <is>
           <t>6 años (Plazo de prescripción tributaria según normas del SII)</t>
         </is>
       </c>
-      <c r="J9" s="12" t="inlineStr">
-        <is>
-          <t>Cifrado TLS/SSL en web, pasarela de pago certificada PCI-DSS compliance</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="55" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="J9" s="17" t="inlineStr">
+        <is>
+          <t>Cifrado TLS/SSL en web, pasarela de pago certificada con estándar PCI-DSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>RAT-05</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Marketing &amp; Comercial</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Nombre, correo electrónico, teléfono celular</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>Prospectos comerciales y clientes registrados</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>Envío de promociones comerciales, novedades del servicio y cotizaciones solicitadas</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Consentimiento previo, expreso e informado del titular (Art. 13 letra c)</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="G10" s="14" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="H10" s="13" t="inlineStr">
         <is>
           <t>Plataforma de Email Marketing / CRM en la nube con contrato DPA firmado</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr">
+      <c r="I10" s="13" t="inlineStr">
         <is>
           <t>Hasta que el titular revoque su consentimiento (Derecho de Oposición ARCOP)</t>
         </is>
       </c>
-      <c r="J10" s="8" t="inlineStr">
+      <c r="J10" s="13" t="inlineStr">
         <is>
           <t>Enlace directo y gratuito de desuscripción automática (opt-out) en cada comunicación</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="55" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="11" ht="54" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>RAT-06</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>Seguridad de Instalaciones</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Seguridad Instalaciones</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>Imágenes y grabaciones de video en circuito cerrado (CCTV)</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>Colaboradores, clientes, proveedores y visitantes</t>
         </is>
       </c>
-      <c r="E11" s="12" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>Seguridad física de las instalaciones, control de accesos y prevención de delitos</t>
         </is>
       </c>
-      <c r="F11" s="12" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>Interés legítimo del responsable en la seguridad patrimonial y física (Art. 13 letra e)</t>
         </is>
       </c>
-      <c r="G11" s="15" t="inlineStr">
+      <c r="G11" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H11" s="12" t="inlineStr">
+      <c r="H11" s="17" t="inlineStr">
         <is>
           <t>Tribunales de Justicia o Ministerio Público (exclusivamente ante orden judicial formal)</t>
         </is>
       </c>
-      <c r="I11" s="12" t="inlineStr">
+      <c r="I11" s="17" t="inlineStr">
         <is>
           <t>30 días continuos (salvo investigación judicial o policial en curso)</t>
         </is>
       </c>
-      <c r="J11" s="12" t="inlineStr">
+      <c r="J11" s="17" t="inlineStr">
         <is>
           <t>Sobreescritura cíclica automática cada 30 días, servidor de video DVR bajo llave física</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>INSTRUCCIONES OFICIALES DE CUMPLIMIENTO (LEY N° 21.719):</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
-        <is>
-          <t>1. Obligatoriedad Legal:</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>Conforme al Artículo 14 ter de la Ley 21.719, toda empresa que trate datos personales debe mantener este inventario actualizado.</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="n"/>
-      <c r="D14" s="19" t="n"/>
-      <c r="E14" s="19" t="n"/>
-      <c r="F14" s="19" t="n"/>
-      <c r="G14" s="19" t="n"/>
-      <c r="H14" s="19" t="n"/>
-      <c r="I14" s="19" t="n"/>
-      <c r="J14" s="19" t="n"/>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
-        <is>
-          <t>2. Exhibición Fiscalizadora:</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>Este documento es lo primero que exige la Agencia de Protección de Datos Personales (APDP) ante una auditoría.</t>
-        </is>
-      </c>
-      <c r="C15" s="19" t="n"/>
-      <c r="D15" s="19" t="n"/>
-      <c r="E15" s="19" t="n"/>
-      <c r="F15" s="19" t="n"/>
-      <c r="G15" s="19" t="n"/>
-      <c r="H15" s="19" t="n"/>
-      <c r="I15" s="19" t="n"/>
-      <c r="J15" s="19" t="n"/>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>3. Sanción por Omisión:</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>No contar con el Registro RAT constituye Infracción Grave (Art. 35 N° 2) sancionable con multa de hasta 10.000 UTM (~ millones de pesos).</t>
-        </is>
-      </c>
-      <c r="C16" s="19" t="n"/>
-      <c r="D16" s="19" t="n"/>
-      <c r="E16" s="19" t="n"/>
-      <c r="F16" s="19" t="n"/>
-      <c r="G16" s="19" t="n"/>
-      <c r="H16" s="19" t="n"/>
-      <c r="I16" s="19" t="n"/>
-      <c r="J16" s="19" t="n"/>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>4. Personalización:</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>Puedes agregar nuevas filas si tu empresa realiza otras actividades de tratamiento (por ejemplo, encuestas o geolocalización GPS).</t>
-        </is>
-      </c>
-      <c r="C17" s="19" t="n"/>
-      <c r="D17" s="19" t="n"/>
-      <c r="E17" s="19" t="n"/>
-      <c r="F17" s="19" t="n"/>
-      <c r="G17" s="19" t="n"/>
-      <c r="H17" s="19" t="n"/>
-      <c r="I17" s="19" t="n"/>
-      <c r="J17" s="19" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="6">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="I3:J3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>